<commit_message>
Add КД change records to the Excel export
New sheet «Изменения» with the title block change columns (Изм., Кол. уч.,
Лист, № докум., Подп., Дата) stored as text. Records are carried over
when exporting again to the same file.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EwsmT1RoQ6HdiMXxWKR68D
</commit_message>
<xml_diff>
--- a/docs/Пример спецификации.xlsx
+++ b/docs/Пример спецификации.xlsx
@@ -8,7 +8,8 @@
   <x:sheets>
     <x:sheet name="Спецификация" sheetId="1" r:id="rId2"/>
     <x:sheet name="Основная надпись" sheetId="2" r:id="rId3"/>
-    <x:sheet name="Как заполнять" sheetId="3" r:id="rId4"/>
+    <x:sheet name="Изменения" sheetId="3" r:id="rId4"/>
+    <x:sheet name="Как заполнять" sheetId="4" r:id="rId5"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Titles" localSheetId="0">Спецификация!1:1</x:definedName>
@@ -194,6 +195,39 @@
     <x:t>Перв. примен.</x:t>
   </x:si>
   <x:si>
+    <x:t>Изм.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Кол. уч.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Лист</x:t>
+  </x:si>
+  <x:si>
+    <x:t>№ докум.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Подп.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Дата</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>АБВГ.12-25</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Петров</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10.25</x:t>
+  </x:si>
+  <x:si>
     <x:t>Как заполнять</x:t>
   </x:si>
   <x:si>
@@ -225,6 +259,21 @@
   </x:si>
   <x:si>
     <x:t>Лист «Основная надпись» — данные для основной надписи (обозначение, наименование, подписи).</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Лист «Изменения» — графы изменений основной надписи (ГОСТ 2.503), одна строка — одна запись, по порядку внесения:</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">  Изм. — порядковый номер изменения; Кол. уч. — количество изменённых участков на листе;</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">  Лист — номер изменённого листа; № докум. — обозначение извещения об изменении; Подп. и Дата — кто и когда внёс.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>При выводе в PDF запись попадает в основную надпись указанного листа (пустой «Лист» — первый лист);</x:t>
+  </x:si>
+  <x:si>
+    <x:t>если записей больше, чем граф в основной надписи, выводятся последние. Ячейки — текстовые, вводите как есть.</x:t>
   </x:si>
   <x:si>
     <x:t>Файл создан аддином InventorGostSpec. Изменения в нём не возвращаются в сборку Inventor.</x:t>
@@ -234,9 +283,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="0" formatCode=""/>
     <x:numFmt numFmtId="164" formatCode="0.###"/>
+    <x:numFmt numFmtId="165" formatCode="@"/>
   </x:numFmts>
   <x:fonts count="6">
     <x:font>
@@ -346,7 +396,7 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="11">
+  <x:cellStyleXfs count="12">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -377,11 +427,14 @@
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -448,6 +501,14 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
@@ -1418,15 +1479,160 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:A15"/>
+  <x:dimension ref="A1:F12"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="7.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="9.710625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12.710625" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24.710625" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18.710625" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12.710625" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:6">
+      <x:c r="A1" s="17" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B1" s="17" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C1" s="17" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D1" s="17" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="E1" s="17" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="F1" s="17" t="s">
+        <x:v>63</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:6">
+      <x:c r="A2" s="18" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B2" s="18" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C2" s="18" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="D2" s="18" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="E2" s="18" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="F2" s="18" t="s">
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:6">
+      <x:c r="A3" s="18"/>
+      <x:c r="B3" s="18"/>
+      <x:c r="C3" s="18"/>
+      <x:c r="D3" s="18"/>
+      <x:c r="E3" s="18"/>
+      <x:c r="F3" s="18"/>
+    </x:row>
+    <x:row r="4" spans="1:6">
+      <x:c r="A4" s="18"/>
+      <x:c r="B4" s="18"/>
+      <x:c r="C4" s="18"/>
+      <x:c r="D4" s="18"/>
+      <x:c r="E4" s="18"/>
+      <x:c r="F4" s="18"/>
+    </x:row>
+    <x:row r="5" spans="1:6">
+      <x:c r="A5" s="18"/>
+      <x:c r="B5" s="18"/>
+      <x:c r="C5" s="18"/>
+      <x:c r="D5" s="18"/>
+      <x:c r="E5" s="18"/>
+      <x:c r="F5" s="18"/>
+    </x:row>
+    <x:row r="6" spans="1:6">
+      <x:c r="A6" s="18"/>
+      <x:c r="B6" s="18"/>
+      <x:c r="C6" s="18"/>
+      <x:c r="D6" s="18"/>
+      <x:c r="E6" s="18"/>
+      <x:c r="F6" s="18"/>
+    </x:row>
+    <x:row r="7" spans="1:6">
+      <x:c r="A7" s="18"/>
+      <x:c r="B7" s="18"/>
+      <x:c r="C7" s="18"/>
+      <x:c r="D7" s="18"/>
+      <x:c r="E7" s="18"/>
+      <x:c r="F7" s="18"/>
+    </x:row>
+    <x:row r="8" spans="1:6">
+      <x:c r="A8" s="18"/>
+      <x:c r="B8" s="18"/>
+      <x:c r="C8" s="18"/>
+      <x:c r="D8" s="18"/>
+      <x:c r="E8" s="18"/>
+      <x:c r="F8" s="18"/>
+    </x:row>
+    <x:row r="9" spans="1:6">
+      <x:c r="A9" s="18"/>
+      <x:c r="B9" s="18"/>
+      <x:c r="C9" s="18"/>
+      <x:c r="D9" s="18"/>
+      <x:c r="E9" s="18"/>
+      <x:c r="F9" s="18"/>
+    </x:row>
+    <x:row r="10" spans="1:6">
+      <x:c r="A10" s="18"/>
+      <x:c r="B10" s="18"/>
+      <x:c r="C10" s="18"/>
+      <x:c r="D10" s="18"/>
+      <x:c r="E10" s="18"/>
+      <x:c r="F10" s="18"/>
+    </x:row>
+    <x:row r="11" spans="1:6">
+      <x:c r="A11" s="18"/>
+      <x:c r="B11" s="18"/>
+      <x:c r="C11" s="18"/>
+      <x:c r="D11" s="18"/>
+      <x:c r="E11" s="18"/>
+      <x:c r="F11" s="18"/>
+    </x:row>
+    <x:row r="12" spans="1:6">
+      <x:c r="A12" s="18"/>
+      <x:c r="B12" s="18"/>
+      <x:c r="C12" s="18"/>
+      <x:c r="D12" s="18"/>
+      <x:c r="E12" s="18"/>
+      <x:c r="F12" s="18"/>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:A21"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="120.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="17" t="s">
-        <x:v>58</x:v>
+      <x:c r="A1" s="19" t="s">
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
@@ -1436,47 +1642,47 @@
     </x:row>
     <x:row r="3" spans="1:1">
       <x:c r="A3" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
       <x:c r="A4" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
       <x:c r="A5" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
       <x:c r="A6" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
       <x:c r="A7" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:1">
       <x:c r="A8" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:1">
       <x:c r="A9" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:1">
       <x:c r="A10" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:1">
       <x:c r="A11" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:1">
@@ -1486,7 +1692,7 @@
     </x:row>
     <x:row r="13" spans="1:1">
       <x:c r="A13" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:1">
@@ -1496,7 +1702,37 @@
     </x:row>
     <x:row r="15" spans="1:1">
       <x:c r="A15" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>80</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" spans="1:1">
+      <x:c r="A16" s="0" t="s">
+        <x:v>81</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:1">
+      <x:c r="A17" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" spans="1:1">
+      <x:c r="A18" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:1">
+      <x:c r="A19" s="0" t="s">
+        <x:v>84</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" spans="1:1">
+      <x:c r="A20" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:1">
+      <x:c r="A21" s="0" t="s">
+        <x:v>85</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Manual blank rows, page breaks and sheet marks in Excel; title fonts
Excel row types «Пустая» and «Новый лист» add a blank line or start a new
PDF sheet; an empty «Текст» row is a blank line. Excel exports are marked
with the PDF sheets (thick line at each boundary, sheet number in a new
«Лист PDF» column) using the same layout and font settings as the tool,
which now has a button and --mark-sheets to refresh the marks after
manual edits. PDF settings moved to the Pdf library for that.

In the title block the organization is 10 mm on one line and the name
height comes from the new «Шрифт наименования, мм» field, which is kept
from the previous Excel file like the change records.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EwsmT1RoQ6HdiMXxWKR68D
</commit_message>
<xml_diff>
--- a/docs/Пример спецификации.xlsx
+++ b/docs/Пример спецификации.xlsx
@@ -195,6 +195,9 @@
     <x:t>Перв. примен.</x:t>
   </x:si>
   <x:si>
+    <x:t>Шрифт наименования, мм</x:t>
+  </x:si>
+  <x:si>
     <x:t>Изм.</x:t>
   </x:si>
   <x:si>
@@ -249,18 +252,45 @@
     <x:t xml:space="preserve">  Текст — строка текста без позиции (в «Наименовании»);</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">  Резерв — пустая строка резервной позиции (номер позиции можно оставить или стереть).</x:t>
+    <x:t xml:space="preserve">  Резерв — свободная строка резервной позиции (номер позиции для справки, в PDF не выводится);</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">  Пустая — пустая строка, добавленная вручную: например, чтобы сдвинуть запись на следующий лист;</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">  Новый лист — следующие строки начинаются с нового листа PDF (сама строка не выводится).</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Колонка «Лист PDF» и жирные линии показывают, где кончается лист PDF. После ручной правки обновите разметку</x:t>
+  </x:si>
+  <x:si>
+    <x:t>кнопкой «Разметить листы в Excel» в утилите PDF (файл Excel должен быть закрыт).</x:t>
   </x:si>
   <x:si>
     <x:t>Пустой «Тип строки» у заполненной строки считается «Изделием», у пустой — пустой строкой.</x:t>
   </x:si>
   <x:si>
+    <x:t>Ручной перенос строки — Alt+Enter внутри ячейки: в PDF текст перенесётся в этом месте (Обозначение, Наименование,</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Примечание; на листе «Основная надпись» — Наименование и Организация). Без него длинный текст сжимается</x:t>
+  </x:si>
+  <x:si>
+    <x:t>до 80 % по ширине, а если не помещается и так — переносится по словам.</x:t>
+  </x:si>
+  <x:si>
     <x:t>«Ед. изм.» выводится вместе с количеством (например, «2,5 м»); для штук оставьте пустым.</x:t>
   </x:si>
   <x:si>
     <x:t>Лист «Основная надпись» — данные для основной надписи (обозначение, наименование, подписи).</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">  «Шрифт наименования, мм» — высота шрифта наименования изделия в основной надписи (2,5; 3,5; 5; 7; 10).</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">  Не помещается — сжимается по ширине и переносится. Организация выводится шрифтом 10 одной строкой.</x:t>
+  </x:si>
+  <x:si>
     <x:t>Лист «Изменения» — графы изменений основной надписи (ГОСТ 2.503), одна строка — одна запись, по порядку внесения:</x:t>
   </x:si>
   <x:si>
@@ -270,25 +300,29 @@
     <x:t xml:space="preserve">  Лист — номер изменённого листа; № докум. — обозначение извещения об изменении; Подп. и Дата — кто и когда внёс.</x:t>
   </x:si>
   <x:si>
-    <x:t>При выводе в PDF запись попадает в основную надпись указанного листа (пустой «Лист» — первый лист);</x:t>
+    <x:t>При выводе в PDF все записи попадают в основную надпись первого листа, а также указанного в «Лист» листа;</x:t>
   </x:si>
   <x:si>
     <x:t>если записей больше, чем граф в основной надписи, выводятся последние. Ячейки — текстовые, вводите как есть.</x:t>
   </x:si>
   <x:si>
     <x:t>Файл создан аддином InventorGostSpec. Изменения в нём не возвращаются в сборку Inventor.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Лист PDF</x:t>
   </x:si>
 </x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="0" formatCode=""/>
     <x:numFmt numFmtId="164" formatCode="0.###"/>
-    <x:numFmt numFmtId="165" formatCode="@"/>
+    <x:numFmt numFmtId="165" formatCode="0.#"/>
+    <x:numFmt numFmtId="166" formatCode="@"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
@@ -336,6 +370,14 @@
       <x:name val="Calibri"/>
       <x:family val="2"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
   </x:fonts>
   <x:fills count="5">
     <x:fill>
@@ -360,7 +402,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="4">
     <x:border diagonalUp="0" diagonalDown="0">
       <x:left style="none">
         <x:color rgb="FF000000"/>
@@ -395,8 +437,42 @@
         <x:color rgb="FF000000"/>
       </x:diagonal>
     </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FFD9DDE3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9DDE3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9DDE3"/>
+      </x:top>
+      <x:bottom style="thick">
+        <x:color rgb="FF1F2937"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none">
+        <x:color rgb="FF000000"/>
+      </x:left>
+      <x:right style="none">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="none">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="thick">
+        <x:color rgb="FF1F2937"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
   </x:borders>
-  <x:cellStyleXfs count="12">
+  <x:cellStyleXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -430,11 +506,32 @@
     <x:xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -503,15 +600,47 @@
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -822,9 +951,10 @@
     <x:col min="7" max="7" width="7.710625" style="1" customWidth="1"/>
     <x:col min="8" max="8" width="8.710625" style="1" customWidth="1"/>
     <x:col min="9" max="9" width="22.710625" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="9.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:9" ht="22" customHeight="1">
+    <x:row r="1" spans="1:10" ht="22" customHeight="1">
       <x:c r="A1" s="2" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -852,8 +982,11 @@
       <x:c r="I1" s="2" t="s">
         <x:v>8</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:9">
+      <x:c r="J1" s="21" t="s">
+        <x:v>96</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:10">
       <x:c r="A2" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -867,8 +1000,11 @@
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
       <x:c r="I2" s="5"/>
-    </x:row>
-    <x:row r="3" spans="1:9">
+      <x:c r="J2" s="22">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:10">
       <x:c r="A3" s="7" t="s">
         <x:v>11</x:v>
       </x:c>
@@ -895,7 +1031,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" spans="1:9">
+    <x:row r="4" spans="1:10">
       <x:c r="A4" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -910,7 +1046,7 @@
       <x:c r="H4" s="4"/>
       <x:c r="I4" s="5"/>
     </x:row>
-    <x:row r="5" spans="1:9">
+    <x:row r="5" spans="1:10">
       <x:c r="A5" s="7" t="s">
         <x:v>11</x:v>
       </x:c>
@@ -939,7 +1075,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" spans="1:9">
+    <x:row r="6" spans="1:10">
       <x:c r="A6" s="7" t="s">
         <x:v>11</x:v>
       </x:c>
@@ -968,7 +1104,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" spans="1:9">
+    <x:row r="7" spans="1:10">
       <x:c r="A7" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
@@ -983,7 +1119,7 @@
       <x:c r="H7" s="11"/>
       <x:c r="I7" s="7"/>
     </x:row>
-    <x:row r="8" spans="1:9">
+    <x:row r="8" spans="1:10">
       <x:c r="A8" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
@@ -998,7 +1134,7 @@
       <x:c r="H8" s="11"/>
       <x:c r="I8" s="7"/>
     </x:row>
-    <x:row r="9" spans="1:9">
+    <x:row r="9" spans="1:10">
       <x:c r="A9" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1013,7 +1149,7 @@
       <x:c r="H9" s="4"/>
       <x:c r="I9" s="5"/>
     </x:row>
-    <x:row r="10" spans="1:9">
+    <x:row r="10" spans="1:10">
       <x:c r="A10" s="7" t="s">
         <x:v>11</x:v>
       </x:c>
@@ -1042,7 +1178,7 @@
         <x:v>27</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" spans="1:9">
+    <x:row r="11" spans="1:10">
       <x:c r="A11" s="7" t="s">
         <x:v>11</x:v>
       </x:c>
@@ -1071,7 +1207,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" spans="1:9">
+    <x:row r="12" spans="1:10">
       <x:c r="A12" s="7" t="s">
         <x:v>11</x:v>
       </x:c>
@@ -1100,7 +1236,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" spans="1:9">
+    <x:row r="13" spans="1:10">
       <x:c r="A13" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
@@ -1115,7 +1251,7 @@
       <x:c r="H13" s="11"/>
       <x:c r="I13" s="7"/>
     </x:row>
-    <x:row r="14" spans="1:9">
+    <x:row r="14" spans="1:10">
       <x:c r="A14" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
@@ -1130,7 +1266,7 @@
       <x:c r="H14" s="11"/>
       <x:c r="I14" s="7"/>
     </x:row>
-    <x:row r="15" spans="1:9">
+    <x:row r="15" spans="1:10">
       <x:c r="A15" s="7" t="s">
         <x:v>22</x:v>
       </x:c>
@@ -1145,7 +1281,7 @@
       <x:c r="H15" s="11"/>
       <x:c r="I15" s="7"/>
     </x:row>
-    <x:row r="16" spans="1:9">
+    <x:row r="16" spans="1:10">
       <x:c r="A16" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1160,7 +1296,7 @@
       <x:c r="H16" s="4"/>
       <x:c r="I16" s="5"/>
     </x:row>
-    <x:row r="17" spans="1:9">
+    <x:row r="17" spans="1:10">
       <x:c r="A17" s="7" t="s">
         <x:v>11</x:v>
       </x:c>
@@ -1189,7 +1325,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" spans="1:9">
+    <x:row r="18" spans="1:10">
       <x:c r="A18" s="7" t="s">
         <x:v>11</x:v>
       </x:c>
@@ -1218,36 +1354,37 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" spans="1:9">
-      <x:c r="A19" s="7" t="s">
+    <x:row r="19" spans="1:10">
+      <x:c r="A19" s="23" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B19" s="8" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C19" s="8" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D19" s="8">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="E19" s="9" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="F19" s="9" t="s">
+      <x:c r="B19" s="24" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C19" s="24" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D19" s="24">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E19" s="25" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="F19" s="25" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="G19" s="10">
+      <x:c r="G19" s="26">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="H19" s="8" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="I19" s="9" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" spans="1:9">
+      <x:c r="H19" s="24" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="I19" s="25" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="J19" s="27"/>
+    </x:row>
+    <x:row r="20" spans="1:10">
       <x:c r="A20" s="12" t="s">
         <x:v>37</x:v>
       </x:c>
@@ -1261,8 +1398,11 @@
       <x:c r="G20" s="13"/>
       <x:c r="H20" s="13"/>
       <x:c r="I20" s="14"/>
-    </x:row>
-    <x:row r="21" spans="1:9">
+      <x:c r="J20" s="22">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:10">
       <x:c r="A21" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1277,7 +1417,7 @@
       <x:c r="H21" s="4"/>
       <x:c r="I21" s="5"/>
     </x:row>
-    <x:row r="22" spans="1:9">
+    <x:row r="22" spans="1:10">
       <x:c r="A22" s="7" t="s">
         <x:v>11</x:v>
       </x:c>
@@ -1306,7 +1446,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" spans="1:9">
+    <x:row r="23" spans="1:10">
       <x:c r="A23" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1321,7 +1461,7 @@
       <x:c r="H23" s="4"/>
       <x:c r="I23" s="5"/>
     </x:row>
-    <x:row r="24" spans="1:9">
+    <x:row r="24" spans="1:10">
       <x:c r="A24" s="7" t="s">
         <x:v>11</x:v>
       </x:c>
@@ -1352,8 +1492,8 @@
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Тип строки" error="Выберите тип из списка: Группа, Раздел, Изделие, Текст, Резерв." promptTitle="" prompt="" sqref="A2:A2000">
-      <x:formula1>"Группа,Раздел,Изделие,Текст,Резерв"</x:formula1>
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Тип строки" error="Выберите тип из списка: Группа, Раздел, Изделие, Текст, Резерв, Пустая, Новый лист." promptTitle="" prompt="" sqref="A2:A2000">
+      <x:formula1>"Группа,Раздел,Изделие,Текст,Резерв,Пустая,Новый лист"</x:formula1>
       <x:formula2/>
     </x:dataValidation>
   </x:dataValidations>
@@ -1370,10 +1510,10 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:B11"/>
+  <x:dimension ref="A1:B12"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18.710625" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24.710625" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="60.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -1463,6 +1603,14 @@
       </x:c>
       <x:c r="B11" s="16" t="s">
         <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:2">
+      <x:c r="A12" s="16" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B12" s="17">
+        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1491,124 +1639,124 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:6">
-      <x:c r="A1" s="17" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="B1" s="17" t="s">
+      <x:c r="A1" s="18" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="C1" s="17" t="s">
+      <x:c r="B1" s="18" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="D1" s="17" t="s">
+      <x:c r="C1" s="18" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="E1" s="17" t="s">
+      <x:c r="D1" s="18" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="F1" s="17" t="s">
+      <x:c r="E1" s="18" t="s">
         <x:v>63</x:v>
       </x:c>
+      <x:c r="F1" s="18" t="s">
+        <x:v>64</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
-      <x:c r="A2" s="18" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="B2" s="18" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C2" s="18" t="s">
+      <x:c r="A2" s="19" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="D2" s="18" t="s">
+      <x:c r="B2" s="19" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C2" s="19" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="E2" s="18" t="s">
+      <x:c r="D2" s="19" t="s">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="F2" s="18" t="s">
+      <x:c r="E2" s="19" t="s">
         <x:v>68</x:v>
       </x:c>
+      <x:c r="F2" s="19" t="s">
+        <x:v>69</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
-      <x:c r="A3" s="18"/>
-      <x:c r="B3" s="18"/>
-      <x:c r="C3" s="18"/>
-      <x:c r="D3" s="18"/>
-      <x:c r="E3" s="18"/>
-      <x:c r="F3" s="18"/>
+      <x:c r="A3" s="19"/>
+      <x:c r="B3" s="19"/>
+      <x:c r="C3" s="19"/>
+      <x:c r="D3" s="19"/>
+      <x:c r="E3" s="19"/>
+      <x:c r="F3" s="19"/>
     </x:row>
     <x:row r="4" spans="1:6">
-      <x:c r="A4" s="18"/>
-      <x:c r="B4" s="18"/>
-      <x:c r="C4" s="18"/>
-      <x:c r="D4" s="18"/>
-      <x:c r="E4" s="18"/>
-      <x:c r="F4" s="18"/>
+      <x:c r="A4" s="19"/>
+      <x:c r="B4" s="19"/>
+      <x:c r="C4" s="19"/>
+      <x:c r="D4" s="19"/>
+      <x:c r="E4" s="19"/>
+      <x:c r="F4" s="19"/>
     </x:row>
     <x:row r="5" spans="1:6">
-      <x:c r="A5" s="18"/>
-      <x:c r="B5" s="18"/>
-      <x:c r="C5" s="18"/>
-      <x:c r="D5" s="18"/>
-      <x:c r="E5" s="18"/>
-      <x:c r="F5" s="18"/>
+      <x:c r="A5" s="19"/>
+      <x:c r="B5" s="19"/>
+      <x:c r="C5" s="19"/>
+      <x:c r="D5" s="19"/>
+      <x:c r="E5" s="19"/>
+      <x:c r="F5" s="19"/>
     </x:row>
     <x:row r="6" spans="1:6">
-      <x:c r="A6" s="18"/>
-      <x:c r="B6" s="18"/>
-      <x:c r="C6" s="18"/>
-      <x:c r="D6" s="18"/>
-      <x:c r="E6" s="18"/>
-      <x:c r="F6" s="18"/>
+      <x:c r="A6" s="19"/>
+      <x:c r="B6" s="19"/>
+      <x:c r="C6" s="19"/>
+      <x:c r="D6" s="19"/>
+      <x:c r="E6" s="19"/>
+      <x:c r="F6" s="19"/>
     </x:row>
     <x:row r="7" spans="1:6">
-      <x:c r="A7" s="18"/>
-      <x:c r="B7" s="18"/>
-      <x:c r="C7" s="18"/>
-      <x:c r="D7" s="18"/>
-      <x:c r="E7" s="18"/>
-      <x:c r="F7" s="18"/>
+      <x:c r="A7" s="19"/>
+      <x:c r="B7" s="19"/>
+      <x:c r="C7" s="19"/>
+      <x:c r="D7" s="19"/>
+      <x:c r="E7" s="19"/>
+      <x:c r="F7" s="19"/>
     </x:row>
     <x:row r="8" spans="1:6">
-      <x:c r="A8" s="18"/>
-      <x:c r="B8" s="18"/>
-      <x:c r="C8" s="18"/>
-      <x:c r="D8" s="18"/>
-      <x:c r="E8" s="18"/>
-      <x:c r="F8" s="18"/>
+      <x:c r="A8" s="19"/>
+      <x:c r="B8" s="19"/>
+      <x:c r="C8" s="19"/>
+      <x:c r="D8" s="19"/>
+      <x:c r="E8" s="19"/>
+      <x:c r="F8" s="19"/>
     </x:row>
     <x:row r="9" spans="1:6">
-      <x:c r="A9" s="18"/>
-      <x:c r="B9" s="18"/>
-      <x:c r="C9" s="18"/>
-      <x:c r="D9" s="18"/>
-      <x:c r="E9" s="18"/>
-      <x:c r="F9" s="18"/>
+      <x:c r="A9" s="19"/>
+      <x:c r="B9" s="19"/>
+      <x:c r="C9" s="19"/>
+      <x:c r="D9" s="19"/>
+      <x:c r="E9" s="19"/>
+      <x:c r="F9" s="19"/>
     </x:row>
     <x:row r="10" spans="1:6">
-      <x:c r="A10" s="18"/>
-      <x:c r="B10" s="18"/>
-      <x:c r="C10" s="18"/>
-      <x:c r="D10" s="18"/>
-      <x:c r="E10" s="18"/>
-      <x:c r="F10" s="18"/>
+      <x:c r="A10" s="19"/>
+      <x:c r="B10" s="19"/>
+      <x:c r="C10" s="19"/>
+      <x:c r="D10" s="19"/>
+      <x:c r="E10" s="19"/>
+      <x:c r="F10" s="19"/>
     </x:row>
     <x:row r="11" spans="1:6">
-      <x:c r="A11" s="18"/>
-      <x:c r="B11" s="18"/>
-      <x:c r="C11" s="18"/>
-      <x:c r="D11" s="18"/>
-      <x:c r="E11" s="18"/>
-      <x:c r="F11" s="18"/>
+      <x:c r="A11" s="19"/>
+      <x:c r="B11" s="19"/>
+      <x:c r="C11" s="19"/>
+      <x:c r="D11" s="19"/>
+      <x:c r="E11" s="19"/>
+      <x:c r="F11" s="19"/>
     </x:row>
     <x:row r="12" spans="1:6">
-      <x:c r="A12" s="18"/>
-      <x:c r="B12" s="18"/>
-      <x:c r="C12" s="18"/>
-      <x:c r="D12" s="18"/>
-      <x:c r="E12" s="18"/>
-      <x:c r="F12" s="18"/>
+      <x:c r="A12" s="19"/>
+      <x:c r="B12" s="19"/>
+      <x:c r="C12" s="19"/>
+      <x:c r="D12" s="19"/>
+      <x:c r="E12" s="19"/>
+      <x:c r="F12" s="19"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -1624,15 +1772,15 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:A21"/>
+  <x:dimension ref="A1:A30"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="120.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:1">
-      <x:c r="A1" s="19" t="s">
-        <x:v>69</x:v>
+      <x:c r="A1" s="20" t="s">
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1">
@@ -1642,97 +1790,142 @@
     </x:row>
     <x:row r="3" spans="1:1">
       <x:c r="A3" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1">
       <x:c r="A4" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1">
       <x:c r="A5" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1">
       <x:c r="A6" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1">
       <x:c r="A7" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:1">
       <x:c r="A8" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:1">
       <x:c r="A9" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:1">
       <x:c r="A10" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:1">
       <x:c r="A11" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:1">
       <x:c r="A12" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:1">
       <x:c r="A13" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:1">
       <x:c r="A14" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:1">
       <x:c r="A15" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:1">
       <x:c r="A16" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:1">
       <x:c r="A17" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:1">
       <x:c r="A18" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:1">
       <x:c r="A19" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:1">
       <x:c r="A20" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:1">
       <x:c r="A21" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>88</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" spans="1:1">
+      <x:c r="A22" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" spans="1:1">
+      <x:c r="A23" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:1">
+      <x:c r="A24" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:1">
+      <x:c r="A25" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:1">
+      <x:c r="A26" s="0" t="s">
+        <x:v>92</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" spans="1:1">
+      <x:c r="A27" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" spans="1:1">
+      <x:c r="A28" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" spans="1:1">
+      <x:c r="A29" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" spans="1:1">
+      <x:c r="A30" s="0" t="s">
+        <x:v>95</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
PDF: font sizes and text compression in settings
Font sizes (table rows, column titles, vertical titles, designation,
name, organization, title block, margin graphs) and the allowed text
compression are stored in pdf.json and edited in the PDF tool window
with a reset to defaults. 0 % turns off automatic wrapping, 100 %
disables compression. The per-document name height in Excel is now
optional and falls back to the settings.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EwsmT1RoQ6HdiMXxWKR68D
</commit_message>
<xml_diff>
--- a/docs/Пример спецификации.xlsx
+++ b/docs/Пример спецификации.xlsx
@@ -273,10 +273,10 @@
     <x:t>Ручной перенос строки — Alt+Enter внутри ячейки: в PDF текст перенесётся в этом месте (Обозначение, Наименование,</x:t>
   </x:si>
   <x:si>
-    <x:t>Примечание; на листе «Основная надпись» — Наименование и Организация). Без него длинный текст сжимается</x:t>
-  </x:si>
-  <x:si>
-    <x:t>до 80 % по ширине, а если не помещается и так — переносится по словам.</x:t>
+    <x:t>Примечание; на листе «Основная надпись» — Наименование). Без него длинный текст сужается по ширине</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(по умолчанию до 80 %, задаётся в утилите PDF), а если не помещается и так — переносится по словам.</x:t>
   </x:si>
   <x:si>
     <x:t>«Ед. изм.» выводится вместе с количеством (например, «2,5 м»); для штук оставьте пустым.</x:t>
@@ -285,10 +285,10 @@
     <x:t>Лист «Основная надпись» — данные для основной надписи (обозначение, наименование, подписи).</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">  «Шрифт наименования, мм» — высота шрифта наименования изделия в основной надписи (2,5; 3,5; 5; 7; 10).</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  Не помещается — сжимается по ширине и переносится. Организация выводится шрифтом 10 одной строкой.</x:t>
+    <x:t xml:space="preserve">  «Шрифт наименования, мм» — высота шрифта наименования изделия для этого документа (2,5; 3,5; 5; 7; 10);</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">  пусто — из настроек утилиты PDF. Остальные размеры шрифтов и допустимое сужение текста задаются в утилите PDF.</x:t>
   </x:si>
   <x:si>
     <x:t>Лист «Изменения» — графы изменений основной надписи (ГОСТ 2.503), одна строка — одна запись, по порядку внесения:</x:t>
@@ -1609,9 +1609,7 @@
       <x:c r="A12" s="16" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="B12" s="17">
-        <x:v>5</x:v>
-      </x:c>
+      <x:c r="B12" s="17"/>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>

</xml_diff>